<commit_message>
Fixe MOtor gasoline imbalance
</commit_message>
<xml_diff>
--- a/data/ecc_supply_to_mcc.xlsx
+++ b/data/ecc_supply_to_mcc.xlsx
@@ -2125,7 +2125,7 @@
         <v>0</v>
       </c>
       <c r="AV13" s="8">
-        <v>5820.73286270896</v>
+        <v>5820.73215535619</v>
       </c>
       <c r="AW13" s="8">
         <v>0</v>
@@ -2137,7 +2137,7 @@
         <v>0</v>
       </c>
       <c r="AZ13" s="8">
-        <v>67354.0211167639</v>
+        <v>67354.02046594</v>
       </c>
       <c r="BA13" s="8">
         <v>0</v>
@@ -2167,7 +2167,7 @@
         <v>0</v>
       </c>
       <c r="BJ13" s="8">
-        <v>3155.64534081533</v>
+        <v>3155.63573488976</v>
       </c>
       <c r="BK13" s="8">
         <v>0</v>
@@ -4132,7 +4132,7 @@
         <v>0</v>
       </c>
       <c r="AU28" s="8">
-        <v>54768.7189038251</v>
+        <v>54768.4671959323</v>
       </c>
       <c r="AV28" s="8">
         <v>0</v>
@@ -5115,7 +5115,7 @@
         <v>0</v>
       </c>
       <c r="BJ35" s="8">
-        <v>4140.47436592437</v>
+        <v>4140.46176213519</v>
       </c>
       <c r="BK35" s="8">
         <v>0</v>
@@ -6217,7 +6217,7 @@
         <v>0</v>
       </c>
       <c r="AV47" s="8">
-        <v>42469.4304457103</v>
+        <v>42469.4252846988</v>
       </c>
       <c r="AW47" s="8">
         <v>0</v>
@@ -6665,7 +6665,7 @@
         <v>0</v>
       </c>
       <c r="AV54" s="8">
-        <v>62501.1156779955</v>
+        <v>62501.108082674</v>
       </c>
       <c r="AW54" s="8">
         <v>0</v>
@@ -6771,7 +6771,7 @@
         <v>0</v>
       </c>
       <c r="BJ55" s="8">
-        <v>86639.6929976091</v>
+        <v>86639.4292625082</v>
       </c>
       <c r="BK55" s="8">
         <v>0</v>
@@ -6832,7 +6832,7 @@
         <v>0</v>
       </c>
       <c r="BI56" s="8">
-        <v>273.730001811503</v>
+        <v>273.729168565133</v>
       </c>
       <c r="BJ56" s="8">
         <v>0</v>
@@ -7061,7 +7061,7 @@
         <v>0</v>
       </c>
       <c r="AZ60" s="8">
-        <v>2369.24361812096</v>
+        <v>2369.24359522759</v>
       </c>
       <c r="BA60" s="8">
         <v>0</v>
@@ -7125,7 +7125,7 @@
         <v>0</v>
       </c>
       <c r="AZ61" s="8">
-        <v>4830.44426252755</v>
+        <v>4830.44421585225</v>
       </c>
       <c r="BA61" s="8">
         <v>0</v>
@@ -7192,7 +7192,7 @@
         <v>0</v>
       </c>
       <c r="BA62" s="8">
-        <v>4830.44426252755</v>
+        <v>4830.44421585225</v>
       </c>
       <c r="BB62" s="8">
         <v>0</v>
@@ -7442,7 +7442,7 @@
         <v>0</v>
       </c>
       <c r="AY66" s="8">
-        <v>10007.2898093626</v>
+        <v>10007.2438175286</v>
       </c>
       <c r="AZ66" s="8">
         <v>0</v>
@@ -7530,7 +7530,7 @@
         <v>0</v>
       </c>
       <c r="BG67" s="8">
-        <v>3605152.28856941</v>
+        <v>3605152.27697659</v>
       </c>
       <c r="BH67" s="8">
         <v>0</v>
@@ -7603,7 +7603,7 @@
         <v>0</v>
       </c>
       <c r="BJ68" s="8">
-        <v>643.118931908693</v>
+        <v>643.116974225897</v>
       </c>
       <c r="BK68" s="8">
         <v>0</v>
@@ -7664,7 +7664,7 @@
         <v>0</v>
       </c>
       <c r="BI69" s="8">
-        <v>643.118931908693</v>
+        <v>643.116974225897</v>
       </c>
       <c r="BJ69" s="8">
         <v>0</v>
@@ -7725,7 +7725,7 @@
         <v>0</v>
       </c>
       <c r="BH70" s="8">
-        <v>184686.529997727</v>
+        <v>184686.52821315</v>
       </c>
       <c r="BI70" s="8">
         <v>0</v>
@@ -7771,7 +7771,7 @@
         <v>0</v>
       </c>
       <c r="BB71" s="8">
-        <v>184686.529997727</v>
+        <v>184686.52821315</v>
       </c>
       <c r="BC71" s="8">
         <v>0</v>
@@ -7814,7 +7814,7 @@
         <v>0</v>
       </c>
       <c r="AU72" s="8">
-        <v>20810.7013079177</v>
+        <v>20810.6056654072</v>
       </c>
       <c r="AV72" s="8">
         <v>0</v>
@@ -7823,13 +7823,13 @@
         <v>0</v>
       </c>
       <c r="AX72" s="8">
-        <v>-0.000000000213697384684882</v>
+        <v>-0.000000000213697311244698</v>
       </c>
       <c r="AY72" s="8">
         <v>0</v>
       </c>
       <c r="AZ72" s="8">
-        <v>3023109.57430779</v>
+        <v>3023109.54509628</v>
       </c>
       <c r="BA72" s="8">
         <v>0</v>
@@ -7881,7 +7881,7 @@
         <v>0</v>
       </c>
       <c r="AV73" s="8">
-        <v>2915788.43397592</v>
+        <v>2915788.07964064</v>
       </c>
       <c r="AW73" s="8">
         <v>0</v>
@@ -7990,7 +7990,7 @@
         <v>0</v>
       </c>
       <c r="BK74" s="8">
-        <v>20456.406189953</v>
+        <v>20456.3121757237</v>
       </c>
     </row>
     <row r="75">
@@ -8131,7 +8131,7 @@
         <v>0</v>
       </c>
       <c r="AT77" s="8">
-        <v>0.0000000000000135419641776167</v>
+        <v>0.0000000000000135420233746064</v>
       </c>
       <c r="AU77" s="8">
         <v>0</v>
@@ -8149,7 +8149,7 @@
         <v>0</v>
       </c>
       <c r="AZ77" s="8">
-        <v>4390.22190228727</v>
+        <v>4390.22185986572</v>
       </c>
       <c r="BA77" s="8">
         <v>0</v>
@@ -8222,7 +8222,7 @@
         <v>0</v>
       </c>
       <c r="BC78" s="8">
-        <v>4368.51223387163</v>
+        <v>4368.51219165986</v>
       </c>
       <c r="BD78" s="8">
         <v>0</v>
@@ -8341,7 +8341,7 @@
         <v>0</v>
       </c>
       <c r="AZ80" s="8">
-        <v>82.0916287907193</v>
+        <v>82.0916279974897</v>
       </c>
       <c r="BA80" s="8">
         <v>0</v>
@@ -8417,7 +8417,7 @@
         <v>0</v>
       </c>
       <c r="BD81" s="8">
-        <v>82.0916287907193</v>
+        <v>82.0916279974897</v>
       </c>
       <c r="BE81" s="8">
         <v>0</v>
@@ -8597,7 +8597,7 @@
         <v>0</v>
       </c>
       <c r="AZ84" s="8">
-        <v>43.2061204161677</v>
+        <v>43.2061199986785</v>
       </c>
       <c r="BA84" s="8">
         <v>0</v>
@@ -8679,7 +8679,7 @@
         <v>0</v>
       </c>
       <c r="BF85" s="8">
-        <v>43.2061204161677</v>
+        <v>43.2061199986785</v>
       </c>
       <c r="BG85" s="8">
         <v>0</v>
@@ -8894,7 +8894,7 @@
         <v>0</v>
       </c>
       <c r="AV91" s="7">
-        <v>42469.4304457103</v>
+        <v>42469.4252846988</v>
       </c>
       <c r="AW91" s="7">
         <v>0</v>
@@ -9398,7 +9398,7 @@
         <v>0</v>
       </c>
       <c r="AV98" s="7">
-        <v>62501.1156779955</v>
+        <v>62501.108082674</v>
       </c>
       <c r="AW98" s="7">
         <v>0</v>
@@ -9512,7 +9512,7 @@
         <v>0</v>
       </c>
       <c r="BJ99" s="7">
-        <v>86639.6929976091</v>
+        <v>86639.4292625082</v>
       </c>
       <c r="BK99" s="7">
         <v>0</v>
@@ -9581,7 +9581,7 @@
         <v>0</v>
       </c>
       <c r="BI100" s="7">
-        <v>273.730001811503</v>
+        <v>273.729168565133</v>
       </c>
       <c r="BJ100" s="7">
         <v>0</v>
@@ -9614,7 +9614,7 @@
         <v>0</v>
       </c>
       <c r="AV101" s="7">
-        <v>5820.73286270896</v>
+        <v>5820.73215535619</v>
       </c>
       <c r="AW101" s="7">
         <v>0</v>
@@ -9626,7 +9626,7 @@
         <v>0</v>
       </c>
       <c r="AZ101" s="7">
-        <v>67354.0211167639</v>
+        <v>67354.02046594</v>
       </c>
       <c r="BA101" s="7">
         <v>0</v>
@@ -9656,7 +9656,7 @@
         <v>0</v>
       </c>
       <c r="BJ101" s="7">
-        <v>3155.64534081533</v>
+        <v>3155.63573488976</v>
       </c>
       <c r="BK101" s="7">
         <v>0</v>
@@ -9842,7 +9842,7 @@
         <v>0</v>
       </c>
       <c r="AZ104" s="7">
-        <v>2369.24361812096</v>
+        <v>2369.24359522759</v>
       </c>
       <c r="BA104" s="7">
         <v>0</v>
@@ -9914,7 +9914,7 @@
         <v>0</v>
       </c>
       <c r="AZ105" s="7">
-        <v>4830.44426252755</v>
+        <v>4830.44421585225</v>
       </c>
       <c r="BA105" s="7">
         <v>0</v>
@@ -9989,7 +9989,7 @@
         <v>0</v>
       </c>
       <c r="BA106" s="7">
-        <v>4830.44426252755</v>
+        <v>4830.44421585225</v>
       </c>
       <c r="BB106" s="7">
         <v>0</v>
@@ -10243,7 +10243,7 @@
         </is>
       </c>
       <c r="BO109" s="2">
-        <v>23.1502244399504</v>
+        <v>22.7134277524042</v>
       </c>
     </row>
     <row r="110">
@@ -10271,7 +10271,7 @@
         <v>0</v>
       </c>
       <c r="AY110" s="7">
-        <v>10007.2898093626</v>
+        <v>10007.2438175286</v>
       </c>
       <c r="AZ110" s="7">
         <v>0</v>
@@ -10367,7 +10367,7 @@
         <v>0</v>
       </c>
       <c r="BG111" s="7">
-        <v>3605152.28856941</v>
+        <v>3605152.27697659</v>
       </c>
       <c r="BH111" s="7">
         <v>0</v>
@@ -10448,7 +10448,7 @@
         <v>0</v>
       </c>
       <c r="BJ112" s="7">
-        <v>643.118931908693</v>
+        <v>643.116974225897</v>
       </c>
       <c r="BK112" s="7">
         <v>0</v>
@@ -10517,7 +10517,7 @@
         <v>0</v>
       </c>
       <c r="BI113" s="7">
-        <v>643.118931908693</v>
+        <v>643.116974225897</v>
       </c>
       <c r="BJ113" s="7">
         <v>0</v>
@@ -10586,7 +10586,7 @@
         <v>0</v>
       </c>
       <c r="BH114" s="7">
-        <v>184686.529997727</v>
+        <v>184686.52821315</v>
       </c>
       <c r="BI114" s="7">
         <v>0</v>
@@ -10640,7 +10640,7 @@
         <v>0</v>
       </c>
       <c r="BB115" s="7">
-        <v>184686.529997727</v>
+        <v>184686.52821315</v>
       </c>
       <c r="BC115" s="7">
         <v>0</v>
@@ -10691,7 +10691,7 @@
         <v>0</v>
       </c>
       <c r="AU116" s="7">
-        <v>75579.4202117428</v>
+        <v>75579.0728613395</v>
       </c>
       <c r="AV116" s="7">
         <v>0</v>
@@ -10700,13 +10700,13 @@
         <v>0</v>
       </c>
       <c r="AX116" s="7">
-        <v>-0.000000000213697384684882</v>
+        <v>-0.000000000213697311244698</v>
       </c>
       <c r="AY116" s="7">
         <v>0</v>
       </c>
       <c r="AZ116" s="7">
-        <v>3023109.57430779</v>
+        <v>3023109.54509628</v>
       </c>
       <c r="BA116" s="7">
         <v>0</v>
@@ -10766,7 +10766,7 @@
         <v>0</v>
       </c>
       <c r="AV117" s="7">
-        <v>2915788.43397592</v>
+        <v>2915788.07964064</v>
       </c>
       <c r="AW117" s="7">
         <v>0</v>
@@ -10883,7 +10883,7 @@
         <v>0</v>
       </c>
       <c r="BK118" s="7">
-        <v>20456.406189953</v>
+        <v>20456.3121757237</v>
       </c>
       <c r="BN118" s="3" t="inlineStr">
         <is>
@@ -11048,7 +11048,7 @@
         <v>0</v>
       </c>
       <c r="AT121" s="7">
-        <v>0.0000000000000135419641776167</v>
+        <v>0.0000000000000135420233746064</v>
       </c>
       <c r="AU121" s="7">
         <v>0</v>
@@ -11066,7 +11066,7 @@
         <v>0</v>
       </c>
       <c r="AZ121" s="7">
-        <v>4390.22190228727</v>
+        <v>4390.22185986572</v>
       </c>
       <c r="BA121" s="7">
         <v>0</v>
@@ -11147,7 +11147,7 @@
         <v>0</v>
       </c>
       <c r="BC122" s="7">
-        <v>4368.51223387163</v>
+        <v>4368.51219165986</v>
       </c>
       <c r="BD122" s="7">
         <v>0</v>
@@ -11240,7 +11240,7 @@
         <v>0</v>
       </c>
       <c r="BJ123" s="7">
-        <v>4140.47436592437</v>
+        <v>4140.46176213519</v>
       </c>
       <c r="BK123" s="7">
         <v>0</v>
@@ -11282,7 +11282,7 @@
         <v>0</v>
       </c>
       <c r="AZ124" s="7">
-        <v>82.0916287907193</v>
+        <v>82.0916279974897</v>
       </c>
       <c r="BA124" s="7">
         <v>0</v>
@@ -11366,7 +11366,7 @@
         <v>0</v>
       </c>
       <c r="BD125" s="7">
-        <v>82.0916287907193</v>
+        <v>82.0916279974897</v>
       </c>
       <c r="BE125" s="7">
         <v>0</v>
@@ -11570,7 +11570,7 @@
         <v>0</v>
       </c>
       <c r="AZ128" s="7">
-        <v>43.2061204161677</v>
+        <v>43.2061199986785</v>
       </c>
       <c r="BA128" s="7">
         <v>0</v>
@@ -11660,7 +11660,7 @@
         <v>0</v>
       </c>
       <c r="BF129" s="7">
-        <v>43.2061204161677</v>
+        <v>43.2061199986785</v>
       </c>
       <c r="BG129" s="7">
         <v>0</v>
@@ -12046,7 +12046,7 @@
         <v>0</v>
       </c>
       <c r="F135" s="7">
-        <v>0.0000000000000020312876105897</v>
+        <v>0.00000000000000203129649010748</v>
       </c>
       <c r="G135" s="7">
         <v>0</v>
@@ -12245,7 +12245,7 @@
         <v>0</v>
       </c>
       <c r="AD136" s="7">
-        <v>15122.9411248116</v>
+        <v>15122.8716222978</v>
       </c>
       <c r="AE136" s="7">
         <v>0</v>
@@ -12366,7 +12366,7 @@
         <v>0</v>
       </c>
       <c r="AB137" s="7">
-        <v>3020758.98009963</v>
+        <v>3020758.61300801</v>
       </c>
       <c r="AC137" s="7">
         <v>0</v>
@@ -12581,7 +12581,7 @@
         <v>0</v>
       </c>
       <c r="O139" s="7">
-        <v>-0.0000000000574814426462061</v>
+        <v>-0.0000000000574814228918805</v>
       </c>
       <c r="P139" s="7">
         <v>0</v>
@@ -12753,7 +12753,7 @@
         <v>0</v>
       </c>
       <c r="AD140" s="7">
-        <v>5333.46506514077</v>
+        <v>5333.44055342533</v>
       </c>
       <c r="AE140" s="7">
         <v>0</v>
@@ -12829,7 +12829,7 @@
         <v>0</v>
       </c>
       <c r="M141" s="7">
-        <v>1032997.84914179</v>
+        <v>1032997.83916021</v>
       </c>
       <c r="N141" s="7">
         <v>0</v>
@@ -12968,7 +12968,7 @@
         <v>0</v>
       </c>
       <c r="Q142" s="7">
-        <v>4830.44426252755</v>
+        <v>4830.44421585225</v>
       </c>
       <c r="R142" s="7">
         <v>0</v>
@@ -13122,7 +13122,7 @@
         <v>0</v>
       </c>
       <c r="Z143" s="7">
-        <v>184686.529997727</v>
+        <v>184686.52821315</v>
       </c>
       <c r="AA143" s="7">
         <v>0</v>
@@ -13270,7 +13270,7 @@
         <v>0</v>
       </c>
       <c r="AG144" s="7">
-        <v>4368.51223387163</v>
+        <v>4368.51219165986</v>
       </c>
       <c r="AH144" s="7">
         <v>0</v>
@@ -13406,7 +13406,7 @@
         <v>0</v>
       </c>
       <c r="AJ145" s="7">
-        <v>82.0916287907193</v>
+        <v>82.0916279974897</v>
       </c>
       <c r="AK145" s="7">
         <v>0</v>
@@ -13672,7 +13672,7 @@
         <v>0</v>
       </c>
       <c r="AN147" s="7">
-        <v>43.2061204161677</v>
+        <v>43.2061199986785</v>
       </c>
       <c r="AO147" s="7">
         <v>0</v>
@@ -13745,7 +13745,7 @@
         <v>0</v>
       </c>
       <c r="V148" s="7">
-        <v>3605152.28856941</v>
+        <v>3605152.27697659</v>
       </c>
       <c r="W148" s="7">
         <v>0</v>
@@ -13845,7 +13845,7 @@
         <v>0</v>
       </c>
       <c r="M149" s="7">
-        <v>60946.5548992509</v>
+        <v>60946.5543103406</v>
       </c>
       <c r="N149" s="7">
         <v>0</v>
@@ -13966,7 +13966,7 @@
         <v>0</v>
       </c>
       <c r="K150" s="7">
-        <v>273.730001811503</v>
+        <v>273.729168565133</v>
       </c>
       <c r="L150" s="7">
         <v>0</v>
@@ -14005,7 +14005,7 @@
         <v>0</v>
       </c>
       <c r="X150" s="7">
-        <v>643.118931908693</v>
+        <v>643.116974225897</v>
       </c>
       <c r="Y150" s="7">
         <v>0</v>
@@ -14108,7 +14108,7 @@
         <v>0</v>
       </c>
       <c r="P151" s="7">
-        <v>56830.5846644188</v>
+        <v>56830.5846529477</v>
       </c>
       <c r="Q151" s="7">
         <v>0</v>
@@ -14123,7 +14123,7 @@
         <v>0</v>
       </c>
       <c r="U151" s="7">
-        <v>13.3720401395176</v>
+        <v>13.1197374953758</v>
       </c>
       <c r="V151" s="7">
         <v>0</v>
@@ -14165,7 +14165,7 @@
         <v>0</v>
       </c>
       <c r="AI151" s="7">
-        <v>4140.47436592437</v>
+        <v>4140.46176213519</v>
       </c>
       <c r="AJ151" s="7">
         <v>0</v>
@@ -14235,7 +14235,7 @@
         <v>0</v>
       </c>
       <c r="P152" s="7">
-        <v>21889.5244052343</v>
+        <v>21889.524400816</v>
       </c>
       <c r="Q152" s="7">
         <v>0</v>
@@ -14250,7 +14250,7 @@
         <v>0</v>
       </c>
       <c r="U152" s="7">
-        <v>5.33289668659379</v>
+        <v>5.23227599439391</v>
       </c>
       <c r="V152" s="7">
         <v>0</v>
@@ -14668,7 +14668,7 @@
         <v>0</v>
       </c>
       <c r="F158" s="2">
-        <v>-0.0000000000000020312876105897</v>
+        <v>-0.00000000000000203129649010748</v>
       </c>
       <c r="G158" s="2">
         <v>0</v>
@@ -14937,7 +14937,7 @@
         <v>0</v>
       </c>
       <c r="K160" s="2">
-        <v>77382.6420272566</v>
+        <v>77382.4064710329</v>
       </c>
       <c r="L160" s="2">
         <v>0</v>
@@ -15070,7 +15070,7 @@
         <v>0</v>
       </c>
       <c r="M161" s="2">
-        <v>40734.7303283613</v>
+        <v>40734.7299347524</v>
       </c>
       <c r="N161" s="2">
         <v>0</v>
@@ -15333,7 +15333,7 @@
         <v>0</v>
       </c>
       <c r="P163" s="2">
-        <v>34699.3669933295</v>
+        <v>34699.3669863255</v>
       </c>
       <c r="Q163" s="2">
         <v>0</v>
@@ -15729,7 +15729,7 @@
         <v>0</v>
       </c>
       <c r="U166" s="2">
-        <v>2.691774313799</v>
+        <v>2.64098611919903</v>
       </c>
       <c r="V166" s="2">
         <v>0</v>
@@ -15859,7 +15859,7 @@
         <v>0</v>
       </c>
       <c r="V167" s="2">
-        <v>10697451.7977645</v>
+        <v>10697451.7633655</v>
       </c>
       <c r="W167" s="2">
         <v>0</v>
@@ -16146,7 +16146,7 @@
         <v>0</v>
       </c>
       <c r="AG169" s="2">
-        <v>21.7096684156417</v>
+        <v>21.7096682058663</v>
       </c>
       <c r="AH169" s="2">
         <v>0</v>
@@ -16183,7 +16183,7 @@
         <v>0</v>
       </c>
       <c r="C170" s="2">
-        <v>42469.4304457103</v>
+        <v>42469.4252846988</v>
       </c>
       <c r="D170" s="2">
         <v>0</v>
@@ -16331,7 +16331,7 @@
         <v>0</v>
       </c>
       <c r="J171" s="2">
-        <v>62501.1156779955</v>
+        <v>62501.108082674</v>
       </c>
       <c r="K171" s="2">
         <v>0</v>
@@ -16464,7 +16464,7 @@
         <v>0</v>
       </c>
       <c r="L172" s="2">
-        <v>273.730001811503</v>
+        <v>273.729168565133</v>
       </c>
       <c r="M172" s="2">
         <v>0</v>
@@ -16609,7 +16609,7 @@
         <v>0</v>
       </c>
       <c r="R173" s="2">
-        <v>4830.44426252755</v>
+        <v>4830.44421585225</v>
       </c>
       <c r="S173" s="2">
         <v>0</v>
@@ -16757,7 +16757,7 @@
         <v>0</v>
       </c>
       <c r="Y174" s="2">
-        <v>643.118931908693</v>
+        <v>643.116974225897</v>
       </c>
       <c r="Z174" s="2">
         <v>0</v>
@@ -16878,7 +16878,7 @@
         <v>0</v>
       </c>
       <c r="W175" s="2">
-        <v>3605152.28856941</v>
+        <v>3605152.27697659</v>
       </c>
       <c r="X175" s="2">
         <v>0</v>
@@ -17017,7 +17017,7 @@
         <v>0</v>
       </c>
       <c r="AA176" s="2">
-        <v>184686.529997727</v>
+        <v>184686.52821315</v>
       </c>
       <c r="AB176" s="2">
         <v>0</v>
@@ -17150,7 +17150,7 @@
         <v>0</v>
       </c>
       <c r="AC177" s="2">
-        <v>2915788.43397592</v>
+        <v>2915788.07964064</v>
       </c>
       <c r="AD177" s="2">
         <v>0</v>
@@ -17292,7 +17292,7 @@
         <v>0</v>
       </c>
       <c r="AH178" s="2">
-        <v>4368.51223387163</v>
+        <v>4368.51219165986</v>
       </c>
       <c r="AI178" s="2">
         <v>0</v>
@@ -17428,7 +17428,7 @@
         <v>0</v>
       </c>
       <c r="AK179" s="2">
-        <v>82.0916287907193</v>
+        <v>82.0916279974897</v>
       </c>
       <c r="AL179" s="2">
         <v>0</v>
@@ -17694,7 +17694,7 @@
         <v>0</v>
       </c>
       <c r="AO181" s="2">
-        <v>43.2061204161677</v>
+        <v>43.2061199986785</v>
       </c>
     </row>
     <row r="182">
@@ -17731,7 +17731,7 @@
         <v>0</v>
       </c>
       <c r="K182" s="2">
-        <v>8386.09187367954</v>
+        <v>8386.06634604076</v>
       </c>
       <c r="L182" s="2">
         <v>0</v>
@@ -17761,7 +17761,7 @@
         <v>0</v>
       </c>
       <c r="U182" s="2">
-        <v>1.75351330004002</v>
+        <v>1.72042814343549</v>
       </c>
       <c r="V182" s="2">
         <v>0</v>
@@ -17782,7 +17782,7 @@
         <v>0</v>
       </c>
       <c r="AB182" s="2">
-        <v>77930.014419904</v>
+        <v>77930.0049496157</v>
       </c>
       <c r="AC182" s="2">
         <v>0</v>
@@ -17858,7 +17858,7 @@
         <v>0</v>
       </c>
       <c r="K183" s="2">
-        <v>597.229094861451</v>
+        <v>597.227276869372</v>
       </c>
       <c r="L183" s="2">
         <v>0</v>

</xml_diff>